<commit_message>
Remove specific building sites from the monthly expense summary
Remove "평택이곡7단지" and "공도디자인시티" from the "미래" company entries in the `monthly_summary.xlsx` file.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 65b4c133-1c29-403a-a908-af2de34cc2d3
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 78bfb4bc-17ac-4a72-8e49-a0de64e9bd35
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/af6b671c-f086-4da8-9571-39668ddf1e8b/65b4c133-1c29-403a-a908-af2de34cc2d3/Il3JLOG
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/monthly_summary.xlsx
+++ b/monthly_summary.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S41"/>
+  <dimension ref="A1:S39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1211,24 +1211,22 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="n">
-        <v>8</v>
-      </c>
+      <c r="A20" t="inlineStr"/>
       <c r="B20" t="inlineStr">
         <is>
           <t>미래</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>평택이곡7단지</t>
+          <t>청담현대3차</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>1199520</v>
+        <v>720000</v>
       </c>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr"/>
@@ -1246,7 +1244,7 @@
         <v>0</v>
       </c>
       <c r="S20" t="n">
-        <v>1199520</v>
+        <v>720000</v>
       </c>
     </row>
     <row r="21">
@@ -1257,11 +1255,11 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>청담현대3차</t>
+          <t>에이엔디전자저울</t>
         </is>
       </c>
       <c r="E21" t="n">
@@ -1294,15 +1292,15 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>공도디자인시티</t>
+          <t>고산센트레빌NHF5단지</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>1680000</v>
+        <v>840000</v>
       </c>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr"/>
@@ -1320,7 +1318,7 @@
         <v>0</v>
       </c>
       <c r="S22" t="n">
-        <v>1680000</v>
+        <v>840000</v>
       </c>
     </row>
     <row r="23">
@@ -1331,15 +1329,15 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>에이엔디전자저울</t>
+          <t>성남메트로칸</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>720000</v>
+        <v>540000</v>
       </c>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr"/>
@@ -1357,7 +1355,7 @@
         <v>0</v>
       </c>
       <c r="S23" t="n">
-        <v>720000</v>
+        <v>540000</v>
       </c>
     </row>
     <row r="24">
@@ -1368,15 +1366,15 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>고산센트레빌NHF5단지</t>
+          <t>능곡풍림아이원</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>840000</v>
+        <v>720000</v>
       </c>
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr"/>
@@ -1394,7 +1392,7 @@
         <v>0</v>
       </c>
       <c r="S24" t="n">
-        <v>840000</v>
+        <v>720000</v>
       </c>
     </row>
     <row r="25">
@@ -1405,15 +1403,15 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>성남메트로칸</t>
+          <t>경기도청옛청사</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>540000</v>
+        <v>1680000</v>
       </c>
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr"/>
@@ -1431,7 +1429,7 @@
         <v>0</v>
       </c>
       <c r="S25" t="n">
-        <v>540000</v>
+        <v>1680000</v>
       </c>
     </row>
     <row r="26">
@@ -1442,15 +1440,15 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>능곡풍림아이원</t>
+          <t>서울교육청학생교육원</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>720000</v>
+        <v>0</v>
       </c>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr"/>
@@ -1468,7 +1466,7 @@
         <v>0</v>
       </c>
       <c r="S26" t="n">
-        <v>720000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
@@ -1479,15 +1477,15 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>경기도청옛청사</t>
+          <t>아주자동차대학교</t>
         </is>
       </c>
       <c r="E27" t="n">
-        <v>1680000</v>
+        <v>0</v>
       </c>
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr"/>
@@ -1505,26 +1503,26 @@
         <v>0</v>
       </c>
       <c r="S27" t="n">
-        <v>1680000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr"/>
       <c r="B28" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>다원</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>27</v>
+        <v>1</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>서울교육청학생교육원</t>
+          <t>브리운스톤쌍문</t>
         </is>
       </c>
       <c r="E28" t="n">
-        <v>0</v>
+        <v>360000</v>
       </c>
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr"/>
@@ -1542,26 +1540,26 @@
         <v>0</v>
       </c>
       <c r="S28" t="n">
-        <v>0</v>
+        <v>360000</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr"/>
       <c r="B29" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>다원</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>28</v>
+        <v>2</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>아주자동차대학교</t>
+          <t>청계벽산</t>
         </is>
       </c>
       <c r="E29" t="n">
-        <v>0</v>
+        <v>480000</v>
       </c>
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr"/>
@@ -1579,7 +1577,7 @@
         <v>0</v>
       </c>
       <c r="S29" t="n">
-        <v>0</v>
+        <v>480000</v>
       </c>
     </row>
     <row r="30">
@@ -1590,15 +1588,15 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>브리운스톤쌍문</t>
+          <t>아양LH5단지</t>
         </is>
       </c>
       <c r="E30" t="n">
-        <v>360000</v>
+        <v>480000</v>
       </c>
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr"/>
@@ -1616,7 +1614,7 @@
         <v>0</v>
       </c>
       <c r="S30" t="n">
-        <v>360000</v>
+        <v>480000</v>
       </c>
     </row>
     <row r="31">
@@ -1627,15 +1625,15 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>청계벽산</t>
+          <t>화성봉담2</t>
         </is>
       </c>
       <c r="E31" t="n">
-        <v>480000</v>
+        <v>600000</v>
       </c>
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr"/>
@@ -1653,7 +1651,7 @@
         <v>0</v>
       </c>
       <c r="S31" t="n">
-        <v>480000</v>
+        <v>600000</v>
       </c>
     </row>
     <row r="32">
@@ -1664,15 +1662,15 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>아양LH5단지</t>
+          <t>SH관악벽산</t>
         </is>
       </c>
       <c r="E32" t="n">
-        <v>480000</v>
+        <v>1800000</v>
       </c>
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr"/>
@@ -1690,7 +1688,7 @@
         <v>0</v>
       </c>
       <c r="S32" t="n">
-        <v>480000</v>
+        <v>1800000</v>
       </c>
     </row>
     <row r="33">
@@ -1701,15 +1699,15 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>화성봉담2</t>
+          <t>SH상계마들</t>
         </is>
       </c>
       <c r="E33" t="n">
-        <v>600000</v>
+        <v>360000</v>
       </c>
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr"/>
@@ -1727,7 +1725,7 @@
         <v>0</v>
       </c>
       <c r="S33" t="n">
-        <v>600000</v>
+        <v>360000</v>
       </c>
     </row>
     <row r="34">
@@ -1738,15 +1736,15 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>SH관악벽산</t>
+          <t>LH당진우강송산</t>
         </is>
       </c>
       <c r="E34" t="n">
-        <v>1800000</v>
+        <v>360000</v>
       </c>
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr"/>
@@ -1764,7 +1762,7 @@
         <v>0</v>
       </c>
       <c r="S34" t="n">
-        <v>1800000</v>
+        <v>360000</v>
       </c>
     </row>
     <row r="35">
@@ -1775,15 +1773,15 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>SH상계마들</t>
+          <t>LH고덕35단지</t>
         </is>
       </c>
       <c r="E35" t="n">
-        <v>360000</v>
+        <v>480000</v>
       </c>
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr"/>
@@ -1801,26 +1799,28 @@
         <v>0</v>
       </c>
       <c r="S35" t="n">
-        <v>360000</v>
+        <v>480000</v>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr"/>
+      <c r="A36" t="n">
+        <v>12</v>
+      </c>
       <c r="B36" t="inlineStr">
         <is>
           <t>다원</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>LH당진우강송산</t>
+          <t>별가람마을1-8단지</t>
         </is>
       </c>
       <c r="E36" t="n">
-        <v>360000</v>
+        <v>720000</v>
       </c>
       <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr"/>
@@ -1838,7 +1838,7 @@
         <v>0</v>
       </c>
       <c r="S36" t="n">
-        <v>360000</v>
+        <v>720000</v>
       </c>
     </row>
     <row r="37">
@@ -1849,15 +1849,15 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>LH고덕35단지</t>
+          <t>남양뉴타운LH19단지</t>
         </is>
       </c>
       <c r="E37" t="n">
-        <v>480000</v>
+        <v>360000</v>
       </c>
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr"/>
@@ -1875,28 +1875,26 @@
         <v>0</v>
       </c>
       <c r="S37" t="n">
+        <v>360000</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr"/>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>다원</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>11</v>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>성남금광</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
         <v>480000</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="n">
-        <v>12</v>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>다원</t>
-        </is>
-      </c>
-      <c r="C38" t="n">
-        <v>9</v>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>별가람마을1-8단지</t>
-        </is>
-      </c>
-      <c r="E38" t="n">
-        <v>720000</v>
       </c>
       <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr"/>
@@ -1914,7 +1912,7 @@
         <v>0</v>
       </c>
       <c r="S38" t="n">
-        <v>720000</v>
+        <v>480000</v>
       </c>
     </row>
     <row r="39">
@@ -1925,15 +1923,15 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>남양뉴타운LH19단지</t>
+          <t>강동리엔파크13단지</t>
         </is>
       </c>
       <c r="E39" t="n">
-        <v>360000</v>
+        <v>960000</v>
       </c>
       <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr"/>
@@ -1951,80 +1949,6 @@
         <v>0</v>
       </c>
       <c r="S39" t="n">
-        <v>360000</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr"/>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>다원</t>
-        </is>
-      </c>
-      <c r="C40" t="n">
-        <v>11</v>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>성남금광</t>
-        </is>
-      </c>
-      <c r="E40" t="n">
-        <v>480000</v>
-      </c>
-      <c r="F40" t="inlineStr"/>
-      <c r="G40" t="inlineStr"/>
-      <c r="H40" t="inlineStr"/>
-      <c r="I40" t="inlineStr"/>
-      <c r="J40" t="inlineStr"/>
-      <c r="K40" t="inlineStr"/>
-      <c r="L40" t="inlineStr"/>
-      <c r="M40" t="inlineStr"/>
-      <c r="N40" t="inlineStr"/>
-      <c r="O40" t="inlineStr"/>
-      <c r="P40" t="inlineStr"/>
-      <c r="Q40" t="inlineStr"/>
-      <c r="R40" t="n">
-        <v>0</v>
-      </c>
-      <c r="S40" t="n">
-        <v>480000</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr"/>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>다원</t>
-        </is>
-      </c>
-      <c r="C41" t="n">
-        <v>13</v>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>강동리엔파크13단지</t>
-        </is>
-      </c>
-      <c r="E41" t="n">
-        <v>960000</v>
-      </c>
-      <c r="F41" t="inlineStr"/>
-      <c r="G41" t="inlineStr"/>
-      <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr"/>
-      <c r="J41" t="inlineStr"/>
-      <c r="K41" t="inlineStr"/>
-      <c r="L41" t="inlineStr"/>
-      <c r="M41" t="inlineStr"/>
-      <c r="N41" t="inlineStr"/>
-      <c r="O41" t="inlineStr"/>
-      <c r="P41" t="inlineStr"/>
-      <c r="Q41" t="inlineStr"/>
-      <c r="R41" t="n">
-        <v>0</v>
-      </c>
-      <c r="S41" t="n">
         <v>960000</v>
       </c>
     </row>
@@ -2039,7 +1963,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S41"/>
+  <dimension ref="A1:S39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2824,24 +2748,22 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="n">
-        <v>8</v>
-      </c>
+      <c r="A20" t="inlineStr"/>
       <c r="B20" t="inlineStr">
         <is>
           <t>미래</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>평택이곡7단지</t>
+          <t>청담현대3차</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>720000</v>
+        <v>1440000</v>
       </c>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr"/>
@@ -2859,7 +2781,7 @@
         <v>0</v>
       </c>
       <c r="S20" t="n">
-        <v>720000</v>
+        <v>1440000</v>
       </c>
     </row>
     <row r="21">
@@ -2870,15 +2792,15 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>청담현대3차</t>
+          <t>에이엔디전자저울</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>1440000</v>
+        <v>1080000</v>
       </c>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr"/>
@@ -2896,7 +2818,7 @@
         <v>0</v>
       </c>
       <c r="S21" t="n">
-        <v>1440000</v>
+        <v>1080000</v>
       </c>
     </row>
     <row r="22">
@@ -2907,15 +2829,15 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>공도디자인시티</t>
+          <t>고산센트레빌NHF5단지</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>1680840</v>
+        <v>3360000</v>
       </c>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr"/>
@@ -2933,7 +2855,7 @@
         <v>0</v>
       </c>
       <c r="S22" t="n">
-        <v>1680840</v>
+        <v>3360000</v>
       </c>
     </row>
     <row r="23">
@@ -2944,15 +2866,15 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>에이엔디전자저울</t>
+          <t>성남메트로칸</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>1080000</v>
+        <v>1260000</v>
       </c>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr"/>
@@ -2970,7 +2892,7 @@
         <v>0</v>
       </c>
       <c r="S23" t="n">
-        <v>1080000</v>
+        <v>1260000</v>
       </c>
     </row>
     <row r="24">
@@ -2981,15 +2903,15 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>고산센트레빌NHF5단지</t>
+          <t>능곡풍림아이원</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>3360000</v>
+        <v>1776000</v>
       </c>
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr"/>
@@ -3007,7 +2929,7 @@
         <v>0</v>
       </c>
       <c r="S24" t="n">
-        <v>3360000</v>
+        <v>1776000</v>
       </c>
     </row>
     <row r="25">
@@ -3018,15 +2940,15 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>성남메트로칸</t>
+          <t>경기도청옛청사</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>1260000</v>
+        <v>0</v>
       </c>
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr"/>
@@ -3044,7 +2966,7 @@
         <v>0</v>
       </c>
       <c r="S25" t="n">
-        <v>1260000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
@@ -3055,15 +2977,15 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>능곡풍림아이원</t>
+          <t>서울교육청학생교육원</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>1776000</v>
+        <v>936000</v>
       </c>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr"/>
@@ -3081,7 +3003,7 @@
         <v>0</v>
       </c>
       <c r="S26" t="n">
-        <v>1776000</v>
+        <v>936000</v>
       </c>
     </row>
     <row r="27">
@@ -3092,11 +3014,11 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>경기도청옛청사</t>
+          <t>아주자동차대학교</t>
         </is>
       </c>
       <c r="E27" t="n">
@@ -3125,19 +3047,19 @@
       <c r="A28" t="inlineStr"/>
       <c r="B28" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>다원</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>27</v>
+        <v>1</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>서울교육청학생교육원</t>
+          <t>브리운스톤쌍문</t>
         </is>
       </c>
       <c r="E28" t="n">
-        <v>936000</v>
+        <v>480000</v>
       </c>
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr"/>
@@ -3155,26 +3077,26 @@
         <v>0</v>
       </c>
       <c r="S28" t="n">
-        <v>936000</v>
+        <v>480000</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr"/>
       <c r="B29" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>다원</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>28</v>
+        <v>2</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>아주자동차대학교</t>
+          <t>청계벽산</t>
         </is>
       </c>
       <c r="E29" t="n">
-        <v>0</v>
+        <v>4800000</v>
       </c>
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr"/>
@@ -3192,7 +3114,7 @@
         <v>0</v>
       </c>
       <c r="S29" t="n">
-        <v>0</v>
+        <v>4800000</v>
       </c>
     </row>
     <row r="30">
@@ -3203,15 +3125,15 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>브리운스톤쌍문</t>
+          <t>아양LH5단지</t>
         </is>
       </c>
       <c r="E30" t="n">
-        <v>480000</v>
+        <v>1120080</v>
       </c>
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr"/>
@@ -3229,7 +3151,7 @@
         <v>0</v>
       </c>
       <c r="S30" t="n">
-        <v>480000</v>
+        <v>1120080</v>
       </c>
     </row>
     <row r="31">
@@ -3240,15 +3162,15 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>청계벽산</t>
+          <t>화성봉담2</t>
         </is>
       </c>
       <c r="E31" t="n">
-        <v>4800000</v>
+        <v>600000</v>
       </c>
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr"/>
@@ -3266,7 +3188,7 @@
         <v>0</v>
       </c>
       <c r="S31" t="n">
-        <v>4800000</v>
+        <v>600000</v>
       </c>
     </row>
     <row r="32">
@@ -3277,15 +3199,15 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>아양LH5단지</t>
+          <t>SH관악벽산</t>
         </is>
       </c>
       <c r="E32" t="n">
-        <v>1120080</v>
+        <v>2376000</v>
       </c>
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr"/>
@@ -3303,7 +3225,7 @@
         <v>0</v>
       </c>
       <c r="S32" t="n">
-        <v>1120080</v>
+        <v>2376000</v>
       </c>
     </row>
     <row r="33">
@@ -3314,15 +3236,15 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>화성봉담2</t>
+          <t>SH상계마들</t>
         </is>
       </c>
       <c r="E33" t="n">
-        <v>600000</v>
+        <v>840000</v>
       </c>
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr"/>
@@ -3340,7 +3262,7 @@
         <v>0</v>
       </c>
       <c r="S33" t="n">
-        <v>600000</v>
+        <v>840000</v>
       </c>
     </row>
     <row r="34">
@@ -3351,15 +3273,15 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>SH관악벽산</t>
+          <t>LH당진우강송산</t>
         </is>
       </c>
       <c r="E34" t="n">
-        <v>2376000</v>
+        <v>600000</v>
       </c>
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr"/>
@@ -3377,7 +3299,7 @@
         <v>0</v>
       </c>
       <c r="S34" t="n">
-        <v>2376000</v>
+        <v>600000</v>
       </c>
     </row>
     <row r="35">
@@ -3388,15 +3310,15 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>SH상계마들</t>
+          <t>LH고덕35단지</t>
         </is>
       </c>
       <c r="E35" t="n">
-        <v>840000</v>
+        <v>768000</v>
       </c>
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr"/>
@@ -3414,26 +3336,28 @@
         <v>0</v>
       </c>
       <c r="S35" t="n">
-        <v>840000</v>
+        <v>768000</v>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr"/>
+      <c r="A36" t="n">
+        <v>12</v>
+      </c>
       <c r="B36" t="inlineStr">
         <is>
           <t>다원</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>LH당진우강송산</t>
+          <t>별가람마을1-8단지</t>
         </is>
       </c>
       <c r="E36" t="n">
-        <v>600000</v>
+        <v>960000</v>
       </c>
       <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr"/>
@@ -3451,7 +3375,7 @@
         <v>0</v>
       </c>
       <c r="S36" t="n">
-        <v>600000</v>
+        <v>960000</v>
       </c>
     </row>
     <row r="37">
@@ -3462,15 +3386,15 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>LH고덕35단지</t>
+          <t>남양뉴타운LH19단지</t>
         </is>
       </c>
       <c r="E37" t="n">
-        <v>768000</v>
+        <v>360000</v>
       </c>
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr"/>
@@ -3488,28 +3412,26 @@
         <v>0</v>
       </c>
       <c r="S37" t="n">
-        <v>768000</v>
+        <v>360000</v>
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="n">
-        <v>12</v>
-      </c>
+      <c r="A38" t="inlineStr"/>
       <c r="B38" t="inlineStr">
         <is>
           <t>다원</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>별가람마을1-8단지</t>
+          <t>성남금광</t>
         </is>
       </c>
       <c r="E38" t="n">
-        <v>960000</v>
+        <v>480000</v>
       </c>
       <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr"/>
@@ -3527,7 +3449,7 @@
         <v>0</v>
       </c>
       <c r="S38" t="n">
-        <v>960000</v>
+        <v>480000</v>
       </c>
     </row>
     <row r="39">
@@ -3538,15 +3460,15 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>남양뉴타운LH19단지</t>
+          <t>강동리엔파크13단지</t>
         </is>
       </c>
       <c r="E39" t="n">
-        <v>360000</v>
+        <v>960000</v>
       </c>
       <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr"/>
@@ -3564,80 +3486,6 @@
         <v>0</v>
       </c>
       <c r="S39" t="n">
-        <v>360000</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr"/>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>다원</t>
-        </is>
-      </c>
-      <c r="C40" t="n">
-        <v>11</v>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>성남금광</t>
-        </is>
-      </c>
-      <c r="E40" t="n">
-        <v>480000</v>
-      </c>
-      <c r="F40" t="inlineStr"/>
-      <c r="G40" t="inlineStr"/>
-      <c r="H40" t="inlineStr"/>
-      <c r="I40" t="inlineStr"/>
-      <c r="J40" t="inlineStr"/>
-      <c r="K40" t="inlineStr"/>
-      <c r="L40" t="inlineStr"/>
-      <c r="M40" t="inlineStr"/>
-      <c r="N40" t="inlineStr"/>
-      <c r="O40" t="inlineStr"/>
-      <c r="P40" t="inlineStr"/>
-      <c r="Q40" t="inlineStr"/>
-      <c r="R40" t="n">
-        <v>0</v>
-      </c>
-      <c r="S40" t="n">
-        <v>480000</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr"/>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>다원</t>
-        </is>
-      </c>
-      <c r="C41" t="n">
-        <v>13</v>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>강동리엔파크13단지</t>
-        </is>
-      </c>
-      <c r="E41" t="n">
-        <v>960000</v>
-      </c>
-      <c r="F41" t="inlineStr"/>
-      <c r="G41" t="inlineStr"/>
-      <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr"/>
-      <c r="J41" t="inlineStr"/>
-      <c r="K41" t="inlineStr"/>
-      <c r="L41" t="inlineStr"/>
-      <c r="M41" t="inlineStr"/>
-      <c r="N41" t="inlineStr"/>
-      <c r="O41" t="inlineStr"/>
-      <c r="P41" t="inlineStr"/>
-      <c r="Q41" t="inlineStr"/>
-      <c r="R41" t="n">
-        <v>0</v>
-      </c>
-      <c r="S41" t="n">
         <v>960000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove specific housing developments from monthly expense summary
Delete records for '경기도청옛청사', '서울교육청학생교육원', '아양LH5단지', and 'SH상계마들' from the monthly summary Excel file.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 65b4c133-1c29-403a-a908-af2de34cc2d3
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 5312a1ed-e3ec-4965-836f-e545630ff070
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/af6b671c-f086-4da8-9571-39668ddf1e8b/65b4c133-1c29-403a-a908-af2de34cc2d3/D4lAwor
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/monthly_summary.xlsx
+++ b/monthly_summary.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S39"/>
+  <dimension ref="A1:S35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1403,15 +1403,15 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>경기도청옛청사</t>
+          <t>아주자동차대학교</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>1680000</v>
+        <v>0</v>
       </c>
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr"/>
@@ -1429,26 +1429,26 @@
         <v>0</v>
       </c>
       <c r="S25" t="n">
-        <v>1680000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr"/>
       <c r="B26" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>다원</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>27</v>
+        <v>1</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>서울교육청학생교육원</t>
+          <t>브리운스톤쌍문</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>0</v>
+        <v>360000</v>
       </c>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr"/>
@@ -1466,26 +1466,26 @@
         <v>0</v>
       </c>
       <c r="S26" t="n">
-        <v>0</v>
+        <v>360000</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr"/>
       <c r="B27" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>다원</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>28</v>
+        <v>2</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>아주자동차대학교</t>
+          <t>청계벽산</t>
         </is>
       </c>
       <c r="E27" t="n">
-        <v>0</v>
+        <v>480000</v>
       </c>
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr"/>
@@ -1503,7 +1503,7 @@
         <v>0</v>
       </c>
       <c r="S27" t="n">
-        <v>0</v>
+        <v>480000</v>
       </c>
     </row>
     <row r="28">
@@ -1514,15 +1514,15 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>브리운스톤쌍문</t>
+          <t>화성봉담2</t>
         </is>
       </c>
       <c r="E28" t="n">
-        <v>360000</v>
+        <v>600000</v>
       </c>
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr"/>
@@ -1540,7 +1540,7 @@
         <v>0</v>
       </c>
       <c r="S28" t="n">
-        <v>360000</v>
+        <v>600000</v>
       </c>
     </row>
     <row r="29">
@@ -1551,15 +1551,15 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>청계벽산</t>
+          <t>SH관악벽산</t>
         </is>
       </c>
       <c r="E29" t="n">
-        <v>480000</v>
+        <v>1800000</v>
       </c>
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr"/>
@@ -1577,7 +1577,7 @@
         <v>0</v>
       </c>
       <c r="S29" t="n">
-        <v>480000</v>
+        <v>1800000</v>
       </c>
     </row>
     <row r="30">
@@ -1588,15 +1588,15 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>아양LH5단지</t>
+          <t>LH당진우강송산</t>
         </is>
       </c>
       <c r="E30" t="n">
-        <v>480000</v>
+        <v>360000</v>
       </c>
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr"/>
@@ -1614,7 +1614,7 @@
         <v>0</v>
       </c>
       <c r="S30" t="n">
-        <v>480000</v>
+        <v>360000</v>
       </c>
     </row>
     <row r="31">
@@ -1625,15 +1625,15 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>화성봉담2</t>
+          <t>LH고덕35단지</t>
         </is>
       </c>
       <c r="E31" t="n">
-        <v>600000</v>
+        <v>480000</v>
       </c>
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr"/>
@@ -1651,26 +1651,28 @@
         <v>0</v>
       </c>
       <c r="S31" t="n">
-        <v>600000</v>
+        <v>480000</v>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr"/>
+      <c r="A32" t="n">
+        <v>12</v>
+      </c>
       <c r="B32" t="inlineStr">
         <is>
           <t>다원</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>SH관악벽산</t>
+          <t>별가람마을1-8단지</t>
         </is>
       </c>
       <c r="E32" t="n">
-        <v>1800000</v>
+        <v>720000</v>
       </c>
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr"/>
@@ -1688,7 +1690,7 @@
         <v>0</v>
       </c>
       <c r="S32" t="n">
-        <v>1800000</v>
+        <v>720000</v>
       </c>
     </row>
     <row r="33">
@@ -1699,11 +1701,11 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>SH상계마들</t>
+          <t>남양뉴타운LH19단지</t>
         </is>
       </c>
       <c r="E33" t="n">
@@ -1736,15 +1738,15 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>LH당진우강송산</t>
+          <t>성남금광</t>
         </is>
       </c>
       <c r="E34" t="n">
-        <v>360000</v>
+        <v>480000</v>
       </c>
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr"/>
@@ -1762,7 +1764,7 @@
         <v>0</v>
       </c>
       <c r="S34" t="n">
-        <v>360000</v>
+        <v>480000</v>
       </c>
     </row>
     <row r="35">
@@ -1773,15 +1775,15 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>LH고덕35단지</t>
+          <t>강동리엔파크13단지</t>
         </is>
       </c>
       <c r="E35" t="n">
-        <v>480000</v>
+        <v>960000</v>
       </c>
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr"/>
@@ -1799,156 +1801,6 @@
         <v>0</v>
       </c>
       <c r="S35" t="n">
-        <v>480000</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="n">
-        <v>12</v>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>다원</t>
-        </is>
-      </c>
-      <c r="C36" t="n">
-        <v>9</v>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>별가람마을1-8단지</t>
-        </is>
-      </c>
-      <c r="E36" t="n">
-        <v>720000</v>
-      </c>
-      <c r="F36" t="inlineStr"/>
-      <c r="G36" t="inlineStr"/>
-      <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr"/>
-      <c r="K36" t="inlineStr"/>
-      <c r="L36" t="inlineStr"/>
-      <c r="M36" t="inlineStr"/>
-      <c r="N36" t="inlineStr"/>
-      <c r="O36" t="inlineStr"/>
-      <c r="P36" t="inlineStr"/>
-      <c r="Q36" t="inlineStr"/>
-      <c r="R36" t="n">
-        <v>0</v>
-      </c>
-      <c r="S36" t="n">
-        <v>720000</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr"/>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>다원</t>
-        </is>
-      </c>
-      <c r="C37" t="n">
-        <v>10</v>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>남양뉴타운LH19단지</t>
-        </is>
-      </c>
-      <c r="E37" t="n">
-        <v>360000</v>
-      </c>
-      <c r="F37" t="inlineStr"/>
-      <c r="G37" t="inlineStr"/>
-      <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr"/>
-      <c r="J37" t="inlineStr"/>
-      <c r="K37" t="inlineStr"/>
-      <c r="L37" t="inlineStr"/>
-      <c r="M37" t="inlineStr"/>
-      <c r="N37" t="inlineStr"/>
-      <c r="O37" t="inlineStr"/>
-      <c r="P37" t="inlineStr"/>
-      <c r="Q37" t="inlineStr"/>
-      <c r="R37" t="n">
-        <v>0</v>
-      </c>
-      <c r="S37" t="n">
-        <v>360000</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr"/>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>다원</t>
-        </is>
-      </c>
-      <c r="C38" t="n">
-        <v>11</v>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>성남금광</t>
-        </is>
-      </c>
-      <c r="E38" t="n">
-        <v>480000</v>
-      </c>
-      <c r="F38" t="inlineStr"/>
-      <c r="G38" t="inlineStr"/>
-      <c r="H38" t="inlineStr"/>
-      <c r="I38" t="inlineStr"/>
-      <c r="J38" t="inlineStr"/>
-      <c r="K38" t="inlineStr"/>
-      <c r="L38" t="inlineStr"/>
-      <c r="M38" t="inlineStr"/>
-      <c r="N38" t="inlineStr"/>
-      <c r="O38" t="inlineStr"/>
-      <c r="P38" t="inlineStr"/>
-      <c r="Q38" t="inlineStr"/>
-      <c r="R38" t="n">
-        <v>0</v>
-      </c>
-      <c r="S38" t="n">
-        <v>480000</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr"/>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>다원</t>
-        </is>
-      </c>
-      <c r="C39" t="n">
-        <v>13</v>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>강동리엔파크13단지</t>
-        </is>
-      </c>
-      <c r="E39" t="n">
-        <v>960000</v>
-      </c>
-      <c r="F39" t="inlineStr"/>
-      <c r="G39" t="inlineStr"/>
-      <c r="H39" t="inlineStr"/>
-      <c r="I39" t="inlineStr"/>
-      <c r="J39" t="inlineStr"/>
-      <c r="K39" t="inlineStr"/>
-      <c r="L39" t="inlineStr"/>
-      <c r="M39" t="inlineStr"/>
-      <c r="N39" t="inlineStr"/>
-      <c r="O39" t="inlineStr"/>
-      <c r="P39" t="inlineStr"/>
-      <c r="Q39" t="inlineStr"/>
-      <c r="R39" t="n">
-        <v>0</v>
-      </c>
-      <c r="S39" t="n">
         <v>960000</v>
       </c>
     </row>
@@ -1963,7 +1815,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S39"/>
+  <dimension ref="A1:S35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2940,11 +2792,11 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>경기도청옛청사</t>
+          <t>아주자동차대학교</t>
         </is>
       </c>
       <c r="E25" t="n">
@@ -2973,19 +2825,19 @@
       <c r="A26" t="inlineStr"/>
       <c r="B26" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>다원</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>27</v>
+        <v>1</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>서울교육청학생교육원</t>
+          <t>브리운스톤쌍문</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>936000</v>
+        <v>480000</v>
       </c>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr"/>
@@ -3003,26 +2855,26 @@
         <v>0</v>
       </c>
       <c r="S26" t="n">
-        <v>936000</v>
+        <v>480000</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr"/>
       <c r="B27" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>다원</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>28</v>
+        <v>2</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>아주자동차대학교</t>
+          <t>청계벽산</t>
         </is>
       </c>
       <c r="E27" t="n">
-        <v>0</v>
+        <v>4800000</v>
       </c>
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr"/>
@@ -3040,7 +2892,7 @@
         <v>0</v>
       </c>
       <c r="S27" t="n">
-        <v>0</v>
+        <v>4800000</v>
       </c>
     </row>
     <row r="28">
@@ -3051,15 +2903,15 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>브리운스톤쌍문</t>
+          <t>화성봉담2</t>
         </is>
       </c>
       <c r="E28" t="n">
-        <v>480000</v>
+        <v>600000</v>
       </c>
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr"/>
@@ -3077,7 +2929,7 @@
         <v>0</v>
       </c>
       <c r="S28" t="n">
-        <v>480000</v>
+        <v>600000</v>
       </c>
     </row>
     <row r="29">
@@ -3088,15 +2940,15 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>청계벽산</t>
+          <t>SH관악벽산</t>
         </is>
       </c>
       <c r="E29" t="n">
-        <v>4800000</v>
+        <v>2376000</v>
       </c>
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr"/>
@@ -3114,7 +2966,7 @@
         <v>0</v>
       </c>
       <c r="S29" t="n">
-        <v>4800000</v>
+        <v>2376000</v>
       </c>
     </row>
     <row r="30">
@@ -3125,15 +2977,15 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>아양LH5단지</t>
+          <t>LH당진우강송산</t>
         </is>
       </c>
       <c r="E30" t="n">
-        <v>1120080</v>
+        <v>600000</v>
       </c>
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr"/>
@@ -3151,7 +3003,7 @@
         <v>0</v>
       </c>
       <c r="S30" t="n">
-        <v>1120080</v>
+        <v>600000</v>
       </c>
     </row>
     <row r="31">
@@ -3162,15 +3014,15 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>화성봉담2</t>
+          <t>LH고덕35단지</t>
         </is>
       </c>
       <c r="E31" t="n">
-        <v>600000</v>
+        <v>768000</v>
       </c>
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr"/>
@@ -3188,26 +3040,28 @@
         <v>0</v>
       </c>
       <c r="S31" t="n">
-        <v>600000</v>
+        <v>768000</v>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr"/>
+      <c r="A32" t="n">
+        <v>12</v>
+      </c>
       <c r="B32" t="inlineStr">
         <is>
           <t>다원</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>SH관악벽산</t>
+          <t>별가람마을1-8단지</t>
         </is>
       </c>
       <c r="E32" t="n">
-        <v>2376000</v>
+        <v>960000</v>
       </c>
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr"/>
@@ -3225,7 +3079,7 @@
         <v>0</v>
       </c>
       <c r="S32" t="n">
-        <v>2376000</v>
+        <v>960000</v>
       </c>
     </row>
     <row r="33">
@@ -3236,15 +3090,15 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>SH상계마들</t>
+          <t>남양뉴타운LH19단지</t>
         </is>
       </c>
       <c r="E33" t="n">
-        <v>840000</v>
+        <v>360000</v>
       </c>
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr"/>
@@ -3262,7 +3116,7 @@
         <v>0</v>
       </c>
       <c r="S33" t="n">
-        <v>840000</v>
+        <v>360000</v>
       </c>
     </row>
     <row r="34">
@@ -3273,15 +3127,15 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>LH당진우강송산</t>
+          <t>성남금광</t>
         </is>
       </c>
       <c r="E34" t="n">
-        <v>600000</v>
+        <v>480000</v>
       </c>
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr"/>
@@ -3299,7 +3153,7 @@
         <v>0</v>
       </c>
       <c r="S34" t="n">
-        <v>600000</v>
+        <v>480000</v>
       </c>
     </row>
     <row r="35">
@@ -3310,15 +3164,15 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>LH고덕35단지</t>
+          <t>강동리엔파크13단지</t>
         </is>
       </c>
       <c r="E35" t="n">
-        <v>768000</v>
+        <v>960000</v>
       </c>
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr"/>
@@ -3336,156 +3190,6 @@
         <v>0</v>
       </c>
       <c r="S35" t="n">
-        <v>768000</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="n">
-        <v>12</v>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>다원</t>
-        </is>
-      </c>
-      <c r="C36" t="n">
-        <v>9</v>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>별가람마을1-8단지</t>
-        </is>
-      </c>
-      <c r="E36" t="n">
-        <v>960000</v>
-      </c>
-      <c r="F36" t="inlineStr"/>
-      <c r="G36" t="inlineStr"/>
-      <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr"/>
-      <c r="K36" t="inlineStr"/>
-      <c r="L36" t="inlineStr"/>
-      <c r="M36" t="inlineStr"/>
-      <c r="N36" t="inlineStr"/>
-      <c r="O36" t="inlineStr"/>
-      <c r="P36" t="inlineStr"/>
-      <c r="Q36" t="inlineStr"/>
-      <c r="R36" t="n">
-        <v>0</v>
-      </c>
-      <c r="S36" t="n">
-        <v>960000</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr"/>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>다원</t>
-        </is>
-      </c>
-      <c r="C37" t="n">
-        <v>10</v>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>남양뉴타운LH19단지</t>
-        </is>
-      </c>
-      <c r="E37" t="n">
-        <v>360000</v>
-      </c>
-      <c r="F37" t="inlineStr"/>
-      <c r="G37" t="inlineStr"/>
-      <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr"/>
-      <c r="J37" t="inlineStr"/>
-      <c r="K37" t="inlineStr"/>
-      <c r="L37" t="inlineStr"/>
-      <c r="M37" t="inlineStr"/>
-      <c r="N37" t="inlineStr"/>
-      <c r="O37" t="inlineStr"/>
-      <c r="P37" t="inlineStr"/>
-      <c r="Q37" t="inlineStr"/>
-      <c r="R37" t="n">
-        <v>0</v>
-      </c>
-      <c r="S37" t="n">
-        <v>360000</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr"/>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>다원</t>
-        </is>
-      </c>
-      <c r="C38" t="n">
-        <v>11</v>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>성남금광</t>
-        </is>
-      </c>
-      <c r="E38" t="n">
-        <v>480000</v>
-      </c>
-      <c r="F38" t="inlineStr"/>
-      <c r="G38" t="inlineStr"/>
-      <c r="H38" t="inlineStr"/>
-      <c r="I38" t="inlineStr"/>
-      <c r="J38" t="inlineStr"/>
-      <c r="K38" t="inlineStr"/>
-      <c r="L38" t="inlineStr"/>
-      <c r="M38" t="inlineStr"/>
-      <c r="N38" t="inlineStr"/>
-      <c r="O38" t="inlineStr"/>
-      <c r="P38" t="inlineStr"/>
-      <c r="Q38" t="inlineStr"/>
-      <c r="R38" t="n">
-        <v>0</v>
-      </c>
-      <c r="S38" t="n">
-        <v>480000</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr"/>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>다원</t>
-        </is>
-      </c>
-      <c r="C39" t="n">
-        <v>13</v>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>강동리엔파크13단지</t>
-        </is>
-      </c>
-      <c r="E39" t="n">
-        <v>960000</v>
-      </c>
-      <c r="F39" t="inlineStr"/>
-      <c r="G39" t="inlineStr"/>
-      <c r="H39" t="inlineStr"/>
-      <c r="I39" t="inlineStr"/>
-      <c r="J39" t="inlineStr"/>
-      <c r="K39" t="inlineStr"/>
-      <c r="L39" t="inlineStr"/>
-      <c r="M39" t="inlineStr"/>
-      <c r="N39" t="inlineStr"/>
-      <c r="O39" t="inlineStr"/>
-      <c r="P39" t="inlineStr"/>
-      <c r="Q39" t="inlineStr"/>
-      <c r="R39" t="n">
-        <v>0</v>
-      </c>
-      <c r="S39" t="n">
         <v>960000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Format monthly summary numbers with thousand separators
Update the monthly summary display in `app.py` to format all numeric columns (except '구분' and '현장명') with thousand separators using `st.column_config.NumberColumn` with the format "%,d".

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 65b4c133-1c29-403a-a908-af2de34cc2d3
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: e2c2c00e-7a9a-4180-a811-cd8014382a16
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/af6b671c-f086-4da8-9571-39668ddf1e8b/65b4c133-1c29-403a-a908-af2de34cc2d3/D4lAwor
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/monthly_summary.xlsx
+++ b/monthly_summary.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S35"/>
+  <dimension ref="A1:S37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1804,6 +1804,128 @@
         <v>960000</v>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>미래</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr"/>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>신월시영</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>84</v>
+      </c>
+      <c r="F36" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" t="n">
+        <v>0</v>
+      </c>
+      <c r="I36" t="n">
+        <v>0</v>
+      </c>
+      <c r="J36" t="n">
+        <v>0</v>
+      </c>
+      <c r="K36" t="n">
+        <v>0</v>
+      </c>
+      <c r="L36" t="n">
+        <v>0</v>
+      </c>
+      <c r="M36" t="n">
+        <v>0</v>
+      </c>
+      <c r="N36" t="n">
+        <v>0</v>
+      </c>
+      <c r="O36" t="n">
+        <v>0</v>
+      </c>
+      <c r="P36" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q36" t="n">
+        <v>0</v>
+      </c>
+      <c r="R36" t="n">
+        <v>0</v>
+      </c>
+      <c r="S36" t="n">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>다원</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr"/>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>공릉1단지</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>3840000</v>
+      </c>
+      <c r="F37" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" t="n">
+        <v>0</v>
+      </c>
+      <c r="H37" t="n">
+        <v>0</v>
+      </c>
+      <c r="I37" t="n">
+        <v>0</v>
+      </c>
+      <c r="J37" t="n">
+        <v>0</v>
+      </c>
+      <c r="K37" t="n">
+        <v>0</v>
+      </c>
+      <c r="L37" t="n">
+        <v>0</v>
+      </c>
+      <c r="M37" t="n">
+        <v>0</v>
+      </c>
+      <c r="N37" t="n">
+        <v>0</v>
+      </c>
+      <c r="O37" t="n">
+        <v>0</v>
+      </c>
+      <c r="P37" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q37" t="n">
+        <v>0</v>
+      </c>
+      <c r="R37" t="n">
+        <v>0</v>
+      </c>
+      <c r="S37" t="n">
+        <v>3840000</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1815,7 +1937,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S35"/>
+  <dimension ref="A1:S37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3193,6 +3315,128 @@
         <v>960000</v>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>미래</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr"/>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>신월시영</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>84</v>
+      </c>
+      <c r="F36" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" t="n">
+        <v>0</v>
+      </c>
+      <c r="I36" t="n">
+        <v>0</v>
+      </c>
+      <c r="J36" t="n">
+        <v>0</v>
+      </c>
+      <c r="K36" t="n">
+        <v>0</v>
+      </c>
+      <c r="L36" t="n">
+        <v>0</v>
+      </c>
+      <c r="M36" t="n">
+        <v>0</v>
+      </c>
+      <c r="N36" t="n">
+        <v>0</v>
+      </c>
+      <c r="O36" t="n">
+        <v>0</v>
+      </c>
+      <c r="P36" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q36" t="n">
+        <v>0</v>
+      </c>
+      <c r="R36" t="n">
+        <v>0</v>
+      </c>
+      <c r="S36" t="n">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>다원</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr"/>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>공릉1단지</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>1920000</v>
+      </c>
+      <c r="F37" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" t="n">
+        <v>0</v>
+      </c>
+      <c r="H37" t="n">
+        <v>0</v>
+      </c>
+      <c r="I37" t="n">
+        <v>0</v>
+      </c>
+      <c r="J37" t="n">
+        <v>0</v>
+      </c>
+      <c r="K37" t="n">
+        <v>0</v>
+      </c>
+      <c r="L37" t="n">
+        <v>0</v>
+      </c>
+      <c r="M37" t="n">
+        <v>0</v>
+      </c>
+      <c r="N37" t="n">
+        <v>0</v>
+      </c>
+      <c r="O37" t="n">
+        <v>0</v>
+      </c>
+      <c r="P37" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q37" t="n">
+        <v>0</v>
+      </c>
+      <c r="R37" t="n">
+        <v>0</v>
+      </c>
+      <c r="S37" t="n">
+        <v>1920000</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add new housing sites and their budgets to the monthly summary report
Add '신월시영' and '공릉1단지' with their respective clothing and security supply budgets to the monthly summary Excel report.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 7a259c36-598a-4807-9d51-7a9e6bedb772
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 51a6c298-e564-4431-88ab-f48f2b8d1dfd
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/monthly_summary.xlsx
+++ b/monthly_summary.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S35"/>
+  <dimension ref="A1:S37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1804,6 +1804,132 @@
         <v>960000</v>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>14</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>미래</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>14</v>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>신월시영</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>84</v>
+      </c>
+      <c r="F36" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" t="n">
+        <v>0</v>
+      </c>
+      <c r="I36" t="n">
+        <v>0</v>
+      </c>
+      <c r="J36" t="n">
+        <v>0</v>
+      </c>
+      <c r="K36" t="n">
+        <v>0</v>
+      </c>
+      <c r="L36" t="n">
+        <v>0</v>
+      </c>
+      <c r="M36" t="n">
+        <v>0</v>
+      </c>
+      <c r="N36" t="n">
+        <v>0</v>
+      </c>
+      <c r="O36" t="n">
+        <v>0</v>
+      </c>
+      <c r="P36" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q36" t="n">
+        <v>0</v>
+      </c>
+      <c r="R36" t="n">
+        <v>0</v>
+      </c>
+      <c r="S36" t="n">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>15</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>다원</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>15</v>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>공릉1단지</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>3840000</v>
+      </c>
+      <c r="F37" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" t="n">
+        <v>0</v>
+      </c>
+      <c r="H37" t="n">
+        <v>0</v>
+      </c>
+      <c r="I37" t="n">
+        <v>0</v>
+      </c>
+      <c r="J37" t="n">
+        <v>0</v>
+      </c>
+      <c r="K37" t="n">
+        <v>0</v>
+      </c>
+      <c r="L37" t="n">
+        <v>0</v>
+      </c>
+      <c r="M37" t="n">
+        <v>0</v>
+      </c>
+      <c r="N37" t="n">
+        <v>0</v>
+      </c>
+      <c r="O37" t="n">
+        <v>0</v>
+      </c>
+      <c r="P37" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q37" t="n">
+        <v>0</v>
+      </c>
+      <c r="R37" t="n">
+        <v>0</v>
+      </c>
+      <c r="S37" t="n">
+        <v>3840000</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1815,7 +1941,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S35"/>
+  <dimension ref="A1:S37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3193,6 +3319,132 @@
         <v>960000</v>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>14</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>미래</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>14</v>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>신월시영</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>84</v>
+      </c>
+      <c r="F36" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" t="n">
+        <v>0</v>
+      </c>
+      <c r="I36" t="n">
+        <v>0</v>
+      </c>
+      <c r="J36" t="n">
+        <v>0</v>
+      </c>
+      <c r="K36" t="n">
+        <v>0</v>
+      </c>
+      <c r="L36" t="n">
+        <v>0</v>
+      </c>
+      <c r="M36" t="n">
+        <v>0</v>
+      </c>
+      <c r="N36" t="n">
+        <v>0</v>
+      </c>
+      <c r="O36" t="n">
+        <v>0</v>
+      </c>
+      <c r="P36" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q36" t="n">
+        <v>0</v>
+      </c>
+      <c r="R36" t="n">
+        <v>0</v>
+      </c>
+      <c r="S36" t="n">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>15</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>다원</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>15</v>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>공릉1단지</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>1920000</v>
+      </c>
+      <c r="F37" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" t="n">
+        <v>0</v>
+      </c>
+      <c r="H37" t="n">
+        <v>0</v>
+      </c>
+      <c r="I37" t="n">
+        <v>0</v>
+      </c>
+      <c r="J37" t="n">
+        <v>0</v>
+      </c>
+      <c r="K37" t="n">
+        <v>0</v>
+      </c>
+      <c r="L37" t="n">
+        <v>0</v>
+      </c>
+      <c r="M37" t="n">
+        <v>0</v>
+      </c>
+      <c r="N37" t="n">
+        <v>0</v>
+      </c>
+      <c r="O37" t="n">
+        <v>0</v>
+      </c>
+      <c r="P37" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q37" t="n">
+        <v>0</v>
+      </c>
+      <c r="R37" t="n">
+        <v>0</v>
+      </c>
+      <c r="S37" t="n">
+        <v>1920000</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update monthly expense tracking with new budget details
Update budget allocations for specific organizations within the monthly expense tracking system.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 7a259c36-598a-4807-9d51-7a9e6bedb772
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 6b869024-847c-4b7f-8d6f-8c5885659374
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/monthly_summary.xlsx
+++ b/monthly_summary.xlsx
@@ -1411,7 +1411,7 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>0</v>
+        <v>600000</v>
       </c>
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr"/>
@@ -1429,7 +1429,7 @@
         <v>0</v>
       </c>
       <c r="S25" t="n">
-        <v>0</v>
+        <v>600000</v>
       </c>
     </row>
     <row r="26">

</xml_diff>

<commit_message>
Update monthly summary with site and budget modifications
Modify monthly_summary.xlsx to remove 신내10단지, add 신월시영 and 공릉1단지 with their respective budgets, and update 아주자동차대학교's budget.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 7a259c36-598a-4807-9d51-7a9e6bedb772
Replit-Commit-Checkpoint-Type: intermediate_checkpoint
Replit-Commit-Event-Id: 5a451083-4db8-4b26-8768-3a3e87a99c84
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/monthly_summary.xlsx
+++ b/monthly_summary.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S37"/>
+  <dimension ref="A1:S36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -713,7 +713,7 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -721,15 +721,15 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>신내10단지</t>
+          <t>민락청구1차</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>1200000</v>
+        <v>1800000</v>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr"/>
@@ -747,28 +747,28 @@
         <v>0</v>
       </c>
       <c r="S7" t="n">
-        <v>1200000</v>
+        <v>1800000</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
+        <v>1</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>미래</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
         <v>8</v>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>미래</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>7</v>
-      </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>민락청구1차</t>
+          <t>서초4단지</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>1800000</v>
+        <v>480000</v>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr"/>
@@ -786,28 +786,26 @@
         <v>0</v>
       </c>
       <c r="S8" t="n">
-        <v>1800000</v>
+        <v>480000</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="n">
-        <v>1</v>
-      </c>
+      <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr">
         <is>
           <t>미래</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>서초4단지</t>
+          <t>별내미리내4-3</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>480000</v>
+        <v>240000</v>
       </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr"/>
@@ -825,7 +823,7 @@
         <v>0</v>
       </c>
       <c r="S9" t="n">
-        <v>480000</v>
+        <v>240000</v>
       </c>
     </row>
     <row r="10">
@@ -836,11 +834,11 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>별내미리내4-3</t>
+          <t>명지해드는터</t>
         </is>
       </c>
       <c r="E10" t="n">
@@ -866,18 +864,20 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr"/>
+      <c r="A11" t="n">
+        <v>11</v>
+      </c>
       <c r="B11" t="inlineStr">
         <is>
           <t>미래</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>명지해드는터</t>
+          <t>다산한신더휴6</t>
         </is>
       </c>
       <c r="E11" t="n">
@@ -904,7 +904,7 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -912,15 +912,15 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>다산한신더휴6</t>
+          <t>다산한신더휴7</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>240000</v>
+        <v>360000</v>
       </c>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr"/>
@@ -938,12 +938,12 @@
         <v>0</v>
       </c>
       <c r="S12" t="n">
-        <v>240000</v>
+        <v>360000</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -951,15 +951,15 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>다산한신더휴7</t>
+          <t>다산한신더휴8</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>360000</v>
+        <v>240000</v>
       </c>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr"/>
@@ -977,12 +977,12 @@
         <v>0</v>
       </c>
       <c r="S13" t="n">
-        <v>360000</v>
+        <v>240000</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -990,15 +990,15 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>다산한신더휴8</t>
+          <t>노을빛1</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>240000</v>
+        <v>720000</v>
       </c>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr"/>
@@ -1016,28 +1016,26 @@
         <v>0</v>
       </c>
       <c r="S14" t="n">
-        <v>240000</v>
+        <v>720000</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="n">
-        <v>13</v>
-      </c>
+      <c r="A15" t="inlineStr"/>
       <c r="B15" t="inlineStr">
         <is>
           <t>미래</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>노을빛1</t>
+          <t>노을빛2</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>720000</v>
+        <v>1440000</v>
       </c>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr"/>
@@ -1055,7 +1053,7 @@
         <v>0</v>
       </c>
       <c r="S15" t="n">
-        <v>720000</v>
+        <v>1440000</v>
       </c>
     </row>
     <row r="16">
@@ -1066,15 +1064,15 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>노을빛2</t>
+          <t>한울4</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>1440000</v>
+        <v>1260000</v>
       </c>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr"/>
@@ -1092,26 +1090,28 @@
         <v>0</v>
       </c>
       <c r="S16" t="n">
-        <v>1440000</v>
+        <v>1260000</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr"/>
+      <c r="A17" t="n">
+        <v>4</v>
+      </c>
       <c r="B17" t="inlineStr">
         <is>
           <t>미래</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>한울4</t>
+          <t>풍동와이2-1</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>1260000</v>
+        <v>480000</v>
       </c>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr"/>
@@ -1129,12 +1129,12 @@
         <v>0</v>
       </c>
       <c r="S17" t="n">
-        <v>1260000</v>
+        <v>480000</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1142,15 +1142,15 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>풍동와이2-1</t>
+          <t>평택배꽃4단지</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>480000</v>
+        <v>1600320</v>
       </c>
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr"/>
@@ -1168,28 +1168,26 @@
         <v>0</v>
       </c>
       <c r="S18" t="n">
-        <v>480000</v>
+        <v>1600320</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="n">
-        <v>6</v>
-      </c>
+      <c r="A19" t="inlineStr"/>
       <c r="B19" t="inlineStr">
         <is>
           <t>미래</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>평택배꽃4단지</t>
+          <t>청담현대3차</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>1600320</v>
+        <v>720000</v>
       </c>
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr"/>
@@ -1207,7 +1205,7 @@
         <v>0</v>
       </c>
       <c r="S19" t="n">
-        <v>1600320</v>
+        <v>720000</v>
       </c>
     </row>
     <row r="20">
@@ -1218,11 +1216,11 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>청담현대3차</t>
+          <t>에이엔디전자저울</t>
         </is>
       </c>
       <c r="E20" t="n">
@@ -1255,15 +1253,15 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>에이엔디전자저울</t>
+          <t>고산센트레빌NHF5단지</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>720000</v>
+        <v>840000</v>
       </c>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr"/>
@@ -1281,7 +1279,7 @@
         <v>0</v>
       </c>
       <c r="S21" t="n">
-        <v>720000</v>
+        <v>840000</v>
       </c>
     </row>
     <row r="22">
@@ -1292,15 +1290,15 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>고산센트레빌NHF5단지</t>
+          <t>성남메트로칸</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>840000</v>
+        <v>540000</v>
       </c>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr"/>
@@ -1318,7 +1316,7 @@
         <v>0</v>
       </c>
       <c r="S22" t="n">
-        <v>840000</v>
+        <v>540000</v>
       </c>
     </row>
     <row r="23">
@@ -1329,15 +1327,15 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>성남메트로칸</t>
+          <t>능곡풍림아이원</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>540000</v>
+        <v>720000</v>
       </c>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr"/>
@@ -1355,7 +1353,7 @@
         <v>0</v>
       </c>
       <c r="S23" t="n">
-        <v>540000</v>
+        <v>720000</v>
       </c>
     </row>
     <row r="24">
@@ -1366,15 +1364,15 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>능곡풍림아이원</t>
+          <t>아주자동차대학교</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>720000</v>
+        <v>600000</v>
       </c>
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr"/>
@@ -1392,26 +1390,26 @@
         <v>0</v>
       </c>
       <c r="S24" t="n">
-        <v>720000</v>
+        <v>600000</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr"/>
       <c r="B25" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>다원</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>아주자동차대학교</t>
+          <t>브리운스톤쌍문</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>600000</v>
+        <v>360000</v>
       </c>
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr"/>
@@ -1429,7 +1427,7 @@
         <v>0</v>
       </c>
       <c r="S25" t="n">
-        <v>600000</v>
+        <v>360000</v>
       </c>
     </row>
     <row r="26">
@@ -1440,15 +1438,15 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>브리운스톤쌍문</t>
+          <t>청계벽산</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>360000</v>
+        <v>480000</v>
       </c>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr"/>
@@ -1466,7 +1464,7 @@
         <v>0</v>
       </c>
       <c r="S26" t="n">
-        <v>360000</v>
+        <v>480000</v>
       </c>
     </row>
     <row r="27">
@@ -1477,15 +1475,15 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>청계벽산</t>
+          <t>화성봉담2</t>
         </is>
       </c>
       <c r="E27" t="n">
-        <v>480000</v>
+        <v>600000</v>
       </c>
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr"/>
@@ -1503,7 +1501,7 @@
         <v>0</v>
       </c>
       <c r="S27" t="n">
-        <v>480000</v>
+        <v>600000</v>
       </c>
     </row>
     <row r="28">
@@ -1514,15 +1512,15 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>화성봉담2</t>
+          <t>SH관악벽산</t>
         </is>
       </c>
       <c r="E28" t="n">
-        <v>600000</v>
+        <v>1800000</v>
       </c>
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr"/>
@@ -1540,7 +1538,7 @@
         <v>0</v>
       </c>
       <c r="S28" t="n">
-        <v>600000</v>
+        <v>1800000</v>
       </c>
     </row>
     <row r="29">
@@ -1551,15 +1549,15 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>SH관악벽산</t>
+          <t>LH당진우강송산</t>
         </is>
       </c>
       <c r="E29" t="n">
-        <v>1800000</v>
+        <v>360000</v>
       </c>
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr"/>
@@ -1577,7 +1575,7 @@
         <v>0</v>
       </c>
       <c r="S29" t="n">
-        <v>1800000</v>
+        <v>360000</v>
       </c>
     </row>
     <row r="30">
@@ -1588,15 +1586,15 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>LH당진우강송산</t>
+          <t>LH고덕35단지</t>
         </is>
       </c>
       <c r="E30" t="n">
-        <v>360000</v>
+        <v>480000</v>
       </c>
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr"/>
@@ -1614,26 +1612,28 @@
         <v>0</v>
       </c>
       <c r="S30" t="n">
-        <v>360000</v>
+        <v>480000</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr"/>
+      <c r="A31" t="n">
+        <v>12</v>
+      </c>
       <c r="B31" t="inlineStr">
         <is>
           <t>다원</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>LH고덕35단지</t>
+          <t>별가람마을1-8단지</t>
         </is>
       </c>
       <c r="E31" t="n">
-        <v>480000</v>
+        <v>720000</v>
       </c>
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr"/>
@@ -1651,28 +1651,26 @@
         <v>0</v>
       </c>
       <c r="S31" t="n">
-        <v>480000</v>
+        <v>720000</v>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="n">
-        <v>12</v>
-      </c>
+      <c r="A32" t="inlineStr"/>
       <c r="B32" t="inlineStr">
         <is>
           <t>다원</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>별가람마을1-8단지</t>
+          <t>남양뉴타운LH19단지</t>
         </is>
       </c>
       <c r="E32" t="n">
-        <v>720000</v>
+        <v>360000</v>
       </c>
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr"/>
@@ -1690,7 +1688,7 @@
         <v>0</v>
       </c>
       <c r="S32" t="n">
-        <v>720000</v>
+        <v>360000</v>
       </c>
     </row>
     <row r="33">
@@ -1701,15 +1699,15 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>남양뉴타운LH19단지</t>
+          <t>성남금광</t>
         </is>
       </c>
       <c r="E33" t="n">
-        <v>360000</v>
+        <v>480000</v>
       </c>
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr"/>
@@ -1727,7 +1725,7 @@
         <v>0</v>
       </c>
       <c r="S33" t="n">
-        <v>360000</v>
+        <v>480000</v>
       </c>
     </row>
     <row r="34">
@@ -1738,15 +1736,15 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>성남금광</t>
+          <t>강동리엔파크13단지</t>
         </is>
       </c>
       <c r="E34" t="n">
-        <v>480000</v>
+        <v>960000</v>
       </c>
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr"/>
@@ -1764,65 +1762,91 @@
         <v>0</v>
       </c>
       <c r="S34" t="n">
-        <v>480000</v>
+        <v>960000</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr"/>
+      <c r="A35" t="n">
+        <v>14</v>
+      </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>다원</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>강동리엔파크13단지</t>
+          <t>신월시영</t>
         </is>
       </c>
       <c r="E35" t="n">
-        <v>960000</v>
-      </c>
-      <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr"/>
-      <c r="K35" t="inlineStr"/>
-      <c r="L35" t="inlineStr"/>
-      <c r="M35" t="inlineStr"/>
-      <c r="N35" t="inlineStr"/>
-      <c r="O35" t="inlineStr"/>
-      <c r="P35" t="inlineStr"/>
-      <c r="Q35" t="inlineStr"/>
+        <v>84</v>
+      </c>
+      <c r="F35" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" t="n">
+        <v>0</v>
+      </c>
+      <c r="H35" t="n">
+        <v>0</v>
+      </c>
+      <c r="I35" t="n">
+        <v>0</v>
+      </c>
+      <c r="J35" t="n">
+        <v>0</v>
+      </c>
+      <c r="K35" t="n">
+        <v>0</v>
+      </c>
+      <c r="L35" t="n">
+        <v>0</v>
+      </c>
+      <c r="M35" t="n">
+        <v>0</v>
+      </c>
+      <c r="N35" t="n">
+        <v>0</v>
+      </c>
+      <c r="O35" t="n">
+        <v>0</v>
+      </c>
+      <c r="P35" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q35" t="n">
+        <v>0</v>
+      </c>
       <c r="R35" t="n">
         <v>0</v>
       </c>
       <c r="S35" t="n">
-        <v>960000</v>
+        <v>84</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>다원</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>신월시영</t>
+          <t>공릉1단지</t>
         </is>
       </c>
       <c r="E36" t="n">
-        <v>84</v>
+        <v>3840000</v>
       </c>
       <c r="F36" t="n">
         <v>0</v>
@@ -1864,69 +1888,6 @@
         <v>0</v>
       </c>
       <c r="S36" t="n">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="n">
-        <v>15</v>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>다원</t>
-        </is>
-      </c>
-      <c r="C37" t="n">
-        <v>15</v>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>공릉1단지</t>
-        </is>
-      </c>
-      <c r="E37" t="n">
-        <v>3840000</v>
-      </c>
-      <c r="F37" t="n">
-        <v>0</v>
-      </c>
-      <c r="G37" t="n">
-        <v>0</v>
-      </c>
-      <c r="H37" t="n">
-        <v>0</v>
-      </c>
-      <c r="I37" t="n">
-        <v>0</v>
-      </c>
-      <c r="J37" t="n">
-        <v>0</v>
-      </c>
-      <c r="K37" t="n">
-        <v>0</v>
-      </c>
-      <c r="L37" t="n">
-        <v>0</v>
-      </c>
-      <c r="M37" t="n">
-        <v>0</v>
-      </c>
-      <c r="N37" t="n">
-        <v>0</v>
-      </c>
-      <c r="O37" t="n">
-        <v>0</v>
-      </c>
-      <c r="P37" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q37" t="n">
-        <v>0</v>
-      </c>
-      <c r="R37" t="n">
-        <v>0</v>
-      </c>
-      <c r="S37" t="n">
         <v>3840000</v>
       </c>
     </row>
@@ -1941,7 +1902,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S37"/>
+  <dimension ref="A1:S36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2228,7 +2189,7 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -2236,15 +2197,15 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>신내10단지</t>
+          <t>민락청구1차</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>1440000</v>
+        <v>1800000</v>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr"/>
@@ -2262,28 +2223,28 @@
         <v>0</v>
       </c>
       <c r="S7" t="n">
-        <v>1440000</v>
+        <v>1800000</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
+        <v>1</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>미래</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
         <v>8</v>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>미래</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>7</v>
-      </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>민락청구1차</t>
+          <t>서초4단지</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>1800000</v>
+        <v>120000</v>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr"/>
@@ -2301,28 +2262,26 @@
         <v>0</v>
       </c>
       <c r="S8" t="n">
-        <v>1800000</v>
+        <v>120000</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="n">
-        <v>1</v>
-      </c>
+      <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr">
         <is>
           <t>미래</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>서초4단지</t>
+          <t>별내미리내4-3</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>120000</v>
+        <v>480000</v>
       </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr"/>
@@ -2340,7 +2299,7 @@
         <v>0</v>
       </c>
       <c r="S9" t="n">
-        <v>120000</v>
+        <v>480000</v>
       </c>
     </row>
     <row r="10">
@@ -2351,11 +2310,11 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>별내미리내4-3</t>
+          <t>명지해드는터</t>
         </is>
       </c>
       <c r="E10" t="n">
@@ -2381,22 +2340,24 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr"/>
+      <c r="A11" t="n">
+        <v>11</v>
+      </c>
       <c r="B11" t="inlineStr">
         <is>
           <t>미래</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>명지해드는터</t>
+          <t>다산한신더휴6</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>480000</v>
+        <v>840000</v>
       </c>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>
@@ -2414,12 +2375,12 @@
         <v>0</v>
       </c>
       <c r="S11" t="n">
-        <v>480000</v>
+        <v>840000</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -2427,15 +2388,15 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>다산한신더휴6</t>
+          <t>다산한신더휴7</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>840000</v>
+        <v>1260000</v>
       </c>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr"/>
@@ -2453,12 +2414,12 @@
         <v>0</v>
       </c>
       <c r="S12" t="n">
-        <v>840000</v>
+        <v>1260000</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -2466,15 +2427,15 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>다산한신더휴7</t>
+          <t>다산한신더휴8</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>1260000</v>
+        <v>840000</v>
       </c>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr"/>
@@ -2492,12 +2453,12 @@
         <v>0</v>
       </c>
       <c r="S13" t="n">
-        <v>1260000</v>
+        <v>840000</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -2505,15 +2466,15 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>다산한신더휴8</t>
+          <t>노을빛1</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>840000</v>
+        <v>2520000</v>
       </c>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr"/>
@@ -2531,28 +2492,26 @@
         <v>0</v>
       </c>
       <c r="S14" t="n">
-        <v>840000</v>
+        <v>2520000</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="n">
-        <v>13</v>
-      </c>
+      <c r="A15" t="inlineStr"/>
       <c r="B15" t="inlineStr">
         <is>
           <t>미래</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>노을빛1</t>
+          <t>노을빛2</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>2520000</v>
+        <v>5040000</v>
       </c>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr"/>
@@ -2570,7 +2529,7 @@
         <v>0</v>
       </c>
       <c r="S15" t="n">
-        <v>2520000</v>
+        <v>5040000</v>
       </c>
     </row>
     <row r="16">
@@ -2581,15 +2540,15 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>노을빛2</t>
+          <t>한울4</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>5040000</v>
+        <v>2520000</v>
       </c>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr"/>
@@ -2607,26 +2566,28 @@
         <v>0</v>
       </c>
       <c r="S16" t="n">
-        <v>5040000</v>
+        <v>2520000</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr"/>
+      <c r="A17" t="n">
+        <v>4</v>
+      </c>
       <c r="B17" t="inlineStr">
         <is>
           <t>미래</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>한울4</t>
+          <t>풍동와이2-1</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>2520000</v>
+        <v>1440000</v>
       </c>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr"/>
@@ -2644,12 +2605,12 @@
         <v>0</v>
       </c>
       <c r="S17" t="n">
-        <v>2520000</v>
+        <v>1440000</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -2657,15 +2618,15 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>풍동와이2-1</t>
+          <t>평택배꽃4단지</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>1440000</v>
+        <v>5280000</v>
       </c>
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr"/>
@@ -2683,28 +2644,26 @@
         <v>0</v>
       </c>
       <c r="S18" t="n">
+        <v>5280000</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr"/>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>미래</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>20</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>청담현대3차</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
         <v>1440000</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="n">
-        <v>6</v>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>미래</t>
-        </is>
-      </c>
-      <c r="C19" t="n">
-        <v>18</v>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>평택배꽃4단지</t>
-        </is>
-      </c>
-      <c r="E19" t="n">
-        <v>5280000</v>
       </c>
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr"/>
@@ -2722,7 +2681,7 @@
         <v>0</v>
       </c>
       <c r="S19" t="n">
-        <v>5280000</v>
+        <v>1440000</v>
       </c>
     </row>
     <row r="20">
@@ -2733,15 +2692,15 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>청담현대3차</t>
+          <t>에이엔디전자저울</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>1440000</v>
+        <v>1080000</v>
       </c>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr"/>
@@ -2759,7 +2718,7 @@
         <v>0</v>
       </c>
       <c r="S20" t="n">
-        <v>1440000</v>
+        <v>1080000</v>
       </c>
     </row>
     <row r="21">
@@ -2770,15 +2729,15 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>에이엔디전자저울</t>
+          <t>고산센트레빌NHF5단지</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>1080000</v>
+        <v>3360000</v>
       </c>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr"/>
@@ -2796,7 +2755,7 @@
         <v>0</v>
       </c>
       <c r="S21" t="n">
-        <v>1080000</v>
+        <v>3360000</v>
       </c>
     </row>
     <row r="22">
@@ -2807,15 +2766,15 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>고산센트레빌NHF5단지</t>
+          <t>성남메트로칸</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>3360000</v>
+        <v>1260000</v>
       </c>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr"/>
@@ -2833,7 +2792,7 @@
         <v>0</v>
       </c>
       <c r="S22" t="n">
-        <v>3360000</v>
+        <v>1260000</v>
       </c>
     </row>
     <row r="23">
@@ -2844,15 +2803,15 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>성남메트로칸</t>
+          <t>능곡풍림아이원</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>1260000</v>
+        <v>1776000</v>
       </c>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr"/>
@@ -2870,7 +2829,7 @@
         <v>0</v>
       </c>
       <c r="S23" t="n">
-        <v>1260000</v>
+        <v>1776000</v>
       </c>
     </row>
     <row r="24">
@@ -2881,15 +2840,15 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>능곡풍림아이원</t>
+          <t>아주자동차대학교</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>1776000</v>
+        <v>0</v>
       </c>
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr"/>
@@ -2907,26 +2866,26 @@
         <v>0</v>
       </c>
       <c r="S24" t="n">
-        <v>1776000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr"/>
       <c r="B25" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>다원</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>아주자동차대학교</t>
+          <t>브리운스톤쌍문</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>0</v>
+        <v>480000</v>
       </c>
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr"/>
@@ -2944,7 +2903,7 @@
         <v>0</v>
       </c>
       <c r="S25" t="n">
-        <v>0</v>
+        <v>480000</v>
       </c>
     </row>
     <row r="26">
@@ -2955,15 +2914,15 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>브리운스톤쌍문</t>
+          <t>청계벽산</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>480000</v>
+        <v>4800000</v>
       </c>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr"/>
@@ -2981,7 +2940,7 @@
         <v>0</v>
       </c>
       <c r="S26" t="n">
-        <v>480000</v>
+        <v>4800000</v>
       </c>
     </row>
     <row r="27">
@@ -2992,15 +2951,15 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>청계벽산</t>
+          <t>화성봉담2</t>
         </is>
       </c>
       <c r="E27" t="n">
-        <v>4800000</v>
+        <v>600000</v>
       </c>
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr"/>
@@ -3018,7 +2977,7 @@
         <v>0</v>
       </c>
       <c r="S27" t="n">
-        <v>4800000</v>
+        <v>600000</v>
       </c>
     </row>
     <row r="28">
@@ -3029,15 +2988,15 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>화성봉담2</t>
+          <t>SH관악벽산</t>
         </is>
       </c>
       <c r="E28" t="n">
-        <v>600000</v>
+        <v>2376000</v>
       </c>
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr"/>
@@ -3055,7 +3014,7 @@
         <v>0</v>
       </c>
       <c r="S28" t="n">
-        <v>600000</v>
+        <v>2376000</v>
       </c>
     </row>
     <row r="29">
@@ -3066,15 +3025,15 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>SH관악벽산</t>
+          <t>LH당진우강송산</t>
         </is>
       </c>
       <c r="E29" t="n">
-        <v>2376000</v>
+        <v>600000</v>
       </c>
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr"/>
@@ -3092,7 +3051,7 @@
         <v>0</v>
       </c>
       <c r="S29" t="n">
-        <v>2376000</v>
+        <v>600000</v>
       </c>
     </row>
     <row r="30">
@@ -3103,15 +3062,15 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>LH당진우강송산</t>
+          <t>LH고덕35단지</t>
         </is>
       </c>
       <c r="E30" t="n">
-        <v>600000</v>
+        <v>768000</v>
       </c>
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr"/>
@@ -3129,26 +3088,28 @@
         <v>0</v>
       </c>
       <c r="S30" t="n">
-        <v>600000</v>
+        <v>768000</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr"/>
+      <c r="A31" t="n">
+        <v>12</v>
+      </c>
       <c r="B31" t="inlineStr">
         <is>
           <t>다원</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>LH고덕35단지</t>
+          <t>별가람마을1-8단지</t>
         </is>
       </c>
       <c r="E31" t="n">
-        <v>768000</v>
+        <v>960000</v>
       </c>
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr"/>
@@ -3166,28 +3127,26 @@
         <v>0</v>
       </c>
       <c r="S31" t="n">
-        <v>768000</v>
+        <v>960000</v>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="n">
-        <v>12</v>
-      </c>
+      <c r="A32" t="inlineStr"/>
       <c r="B32" t="inlineStr">
         <is>
           <t>다원</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>별가람마을1-8단지</t>
+          <t>남양뉴타운LH19단지</t>
         </is>
       </c>
       <c r="E32" t="n">
-        <v>960000</v>
+        <v>360000</v>
       </c>
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr"/>
@@ -3205,7 +3164,7 @@
         <v>0</v>
       </c>
       <c r="S32" t="n">
-        <v>960000</v>
+        <v>360000</v>
       </c>
     </row>
     <row r="33">
@@ -3216,15 +3175,15 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>남양뉴타운LH19단지</t>
+          <t>성남금광</t>
         </is>
       </c>
       <c r="E33" t="n">
-        <v>360000</v>
+        <v>480000</v>
       </c>
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr"/>
@@ -3242,7 +3201,7 @@
         <v>0</v>
       </c>
       <c r="S33" t="n">
-        <v>360000</v>
+        <v>480000</v>
       </c>
     </row>
     <row r="34">
@@ -3253,15 +3212,15 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>성남금광</t>
+          <t>강동리엔파크13단지</t>
         </is>
       </c>
       <c r="E34" t="n">
-        <v>480000</v>
+        <v>960000</v>
       </c>
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr"/>
@@ -3279,65 +3238,91 @@
         <v>0</v>
       </c>
       <c r="S34" t="n">
-        <v>480000</v>
+        <v>960000</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr"/>
+      <c r="A35" t="n">
+        <v>14</v>
+      </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>다원</t>
+          <t>미래</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>강동리엔파크13단지</t>
+          <t>신월시영</t>
         </is>
       </c>
       <c r="E35" t="n">
-        <v>960000</v>
-      </c>
-      <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr"/>
-      <c r="K35" t="inlineStr"/>
-      <c r="L35" t="inlineStr"/>
-      <c r="M35" t="inlineStr"/>
-      <c r="N35" t="inlineStr"/>
-      <c r="O35" t="inlineStr"/>
-      <c r="P35" t="inlineStr"/>
-      <c r="Q35" t="inlineStr"/>
+        <v>84</v>
+      </c>
+      <c r="F35" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" t="n">
+        <v>0</v>
+      </c>
+      <c r="H35" t="n">
+        <v>0</v>
+      </c>
+      <c r="I35" t="n">
+        <v>0</v>
+      </c>
+      <c r="J35" t="n">
+        <v>0</v>
+      </c>
+      <c r="K35" t="n">
+        <v>0</v>
+      </c>
+      <c r="L35" t="n">
+        <v>0</v>
+      </c>
+      <c r="M35" t="n">
+        <v>0</v>
+      </c>
+      <c r="N35" t="n">
+        <v>0</v>
+      </c>
+      <c r="O35" t="n">
+        <v>0</v>
+      </c>
+      <c r="P35" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q35" t="n">
+        <v>0</v>
+      </c>
       <c r="R35" t="n">
         <v>0</v>
       </c>
       <c r="S35" t="n">
-        <v>960000</v>
+        <v>84</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>미래</t>
+          <t>다원</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>신월시영</t>
+          <t>공릉1단지</t>
         </is>
       </c>
       <c r="E36" t="n">
-        <v>84</v>
+        <v>1920000</v>
       </c>
       <c r="F36" t="n">
         <v>0</v>
@@ -3379,69 +3364,6 @@
         <v>0</v>
       </c>
       <c r="S36" t="n">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="n">
-        <v>15</v>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>다원</t>
-        </is>
-      </c>
-      <c r="C37" t="n">
-        <v>15</v>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>공릉1단지</t>
-        </is>
-      </c>
-      <c r="E37" t="n">
-        <v>1920000</v>
-      </c>
-      <c r="F37" t="n">
-        <v>0</v>
-      </c>
-      <c r="G37" t="n">
-        <v>0</v>
-      </c>
-      <c r="H37" t="n">
-        <v>0</v>
-      </c>
-      <c r="I37" t="n">
-        <v>0</v>
-      </c>
-      <c r="J37" t="n">
-        <v>0</v>
-      </c>
-      <c r="K37" t="n">
-        <v>0</v>
-      </c>
-      <c r="L37" t="n">
-        <v>0</v>
-      </c>
-      <c r="M37" t="n">
-        <v>0</v>
-      </c>
-      <c r="N37" t="n">
-        <v>0</v>
-      </c>
-      <c r="O37" t="n">
-        <v>0</v>
-      </c>
-      <c r="P37" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q37" t="n">
-        <v>0</v>
-      </c>
-      <c r="R37" t="n">
-        <v>0</v>
-      </c>
-      <c r="S37" t="n">
         <v>1920000</v>
       </c>
     </row>

</xml_diff>